<commit_message>
Branch Ops: penyaring Status TBO, cari di Beranda, wajib ganti sandi, sumber dana dan tujuan transfer, penyeragaman ejaan
</commit_message>
<xml_diff>
--- a/contoh/Template-02-Pencairan-Deposito.xlsx
+++ b/contoh/Template-02-Pencairan-Deposito.xlsx
@@ -637,7 +637,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Pemindahbukuan</t>
+          <t>Pemindah-bukuan</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Dipercepat dari Jatuh Tempo</t>
+          <t>Dipercepat (Break)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Pemindahbukuan</t>
+          <t>Pemindah-bukuan</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Dipercepat dari Jatuh Tempo</t>
+          <t>Dipercepat (Break)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -980,6 +980,14 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="K4:K500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Jenis Pencairan tidak dikenal" error="Nilai tidak dikenal. Pilih salah satu dari daftar - ejaan yang berbeda akan membuat baris ini tidak terhitung di dashboard." promptTitle="Jenis Pencairan" prompt="Pilih dari daftar: Sesuai Jatuh Tempo / Dipercepat (Break)" type="list">
+      <formula1>"Sesuai Jatuh Tempo,Dipercepat (Break)"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L4:L500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Jenis Penarikan tidak dikenal" error="Nilai tidak dikenal. Pilih salah satu dari daftar - ejaan yang berbeda akan membuat baris ini tidak terhitung di dashboard." promptTitle="Jenis Penarikan" prompt="Pilih dari daftar: Transfer / Tunai / Pemindah-bukuan" type="list">
+      <formula1>"Transfer,Tunai,Pemindah-bukuan"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>